<commit_message>
Add PLATFORM_REVENUE.md: self-channel strategy as revenue line R5 and sales channel
Adopt both roles for platform (YouTube/TikTok/Niconico) revenue:
- R5 revenue line, capped at 5% of sales, converted to tie-ups (R1/R2) above that
- Sales credibility channel, justified by close-rate improvement not ad revenue
- Third return: retention-rate data that client work cannot produce

Budget model rebuilt with two channel-investment rows in fixed costs:
fixed costs 226 -> 271万, break-even 8.7 -> 10.4 units/month,
recommended funding 3,180 -> 3,643万. 0 formula errors after recalc.

Also: patent-safe publication policy, 4 new China contract clauses,
separate channel production pool, kill criteria at 6 months.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017HoWLm426zeXirBWkACG6e
</commit_message>
<xml_diff>
--- a/budget_model.xlsx
+++ b/budget_model.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="前提" sheetId="1" state="visible" r:id="rId3"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="202">
   <si>
     <r>
       <rPr>
@@ -2250,6 +2250,242 @@
     <t xml:space="preserve">損害賠償責任保険</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">自社チャンネル投資</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(P2: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月開始。営業実績づくり </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">市場反応データ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(PLATFORM_REVENUE.md)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">自社チャンネル投資</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(P3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">拡大分</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2027</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月に月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">本へ拡大。上記と合わせて月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">45</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万になる</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">フル体制での月次固定費</t>
   </si>
   <si>
@@ -2317,6 +2553,55 @@
       </rPr>
       <t xml:space="preserve">平均単価</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">うち 自社チャンネル投資</t>
+  </si>
+  <si>
+    <t xml:space="preserve">営業のための投資。上の損益分岐にはこれも含まれています</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">損益分岐 月間本数</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">チャンネル投資を除く</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">チャンネルを止めた場合の損益分岐。撤退判断のときに見る数字</t>
   </si>
   <si>
     <r>
@@ -5191,7 +5476,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
@@ -5534,48 +5819,120 @@
       <c r="G17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20" t="s">
+      <c r="A18" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C18" s="24" t="n">
-        <f aca="false">SUM(C5:C17)</f>
-        <v>166</v>
-      </c>
-      <c r="D18" s="24" t="n">
-        <f aca="false">SUM(D5:D17)</f>
-        <v>229</v>
-      </c>
-      <c r="E18" s="24" t="n">
-        <f aca="false">SUM(E5:E17)</f>
-        <v>226</v>
-      </c>
-      <c r="F18" s="24" t="n">
-        <f aca="false">SUM(F5:F17)</f>
-        <v>226</v>
+      <c r="B18" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F18" s="22" t="n">
+        <f aca="false">INDEX(C18:E18,前提!$B$11)</f>
+        <v>20</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="F19" s="22" t="n">
+        <f aca="false">INDEX(C19:E19,前提!$B$11)</f>
+        <v>25</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="F20" s="25" t="n">
-        <f aca="false">F18/前提!$E$34</f>
-        <v>417.230769230769</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="F21" s="26" t="n">
-        <f aca="false">F20/前提!$B$21</f>
+        <v>108</v>
+      </c>
+      <c r="C20" s="24" t="n">
+        <f aca="false">SUM(C5:C19)</f>
+        <v>211</v>
+      </c>
+      <c r="D20" s="24" t="n">
+        <f aca="false">SUM(D5:D19)</f>
+        <v>274</v>
+      </c>
+      <c r="E20" s="24" t="n">
+        <f aca="false">SUM(E5:E19)</f>
+        <v>271</v>
+      </c>
+      <c r="F20" s="24" t="n">
+        <f aca="false">SUM(F5:F19)</f>
+        <v>271</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="F22" s="25" t="n">
+        <f aca="false">F20/前提!$E$34</f>
+        <v>500.307692307692</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="F23" s="26" t="n">
+        <f aca="false">F22/前提!$B$21</f>
+        <v>10.4230769230769</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="F25" s="25" t="n">
+        <f aca="false">SUM(F18:F19)</f>
+        <v>45</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="F26" s="26" t="n">
+        <f aca="false">(F20-F25)/前提!$E$34/前提!$B$21</f>
         <v>8.69230769230769</v>
       </c>
-      <c r="G21" s="2" t="s">
-        <v>108</v>
+      <c r="G26" s="2" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -5604,17 +5961,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="20" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B4" s="27" t="n">
         <v>1</v>
@@ -5655,48 +6012,48 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="20" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="B5" s="27" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="E5" s="27" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="F5" s="27" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G5" s="27" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H5" s="27" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="I5" s="27" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="J5" s="27" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="M5" s="27" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="20" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B6" s="28" t="n">
         <v>0</v>
@@ -5735,12 +6092,12 @@
         <v>5</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B7" s="29" t="n">
         <f aca="false">B6*前提!$B$21</f>
@@ -5793,7 +6150,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B9" s="29" t="n">
         <v>0</v>
@@ -5845,7 +6202,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B10" s="22" t="n">
         <f aca="false">前提!$B$14</f>
@@ -5887,7 +6244,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">IF(B4=前提!$B$16,前提!$B$15,0)</f>
@@ -5940,7 +6297,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="B12" s="23" t="n">
         <f aca="false">SUM(B9:B11)</f>
@@ -5993,7 +6350,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="B14" s="22" t="n">
         <f aca="false">SUMIF(初期費用!$B$5:$B$17,B4,初期費用!$F$5:$F$17)</f>
@@ -6046,60 +6403,60 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;B4,月次固定費!$F$5:$F$17)</f>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;B4,月次固定費!$F$5:$F$19)</f>
         <v>56</v>
       </c>
       <c r="C15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;C4,月次固定費!$F$5:$F$17)</f>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;C4,月次固定費!$F$5:$F$19)</f>
         <v>56</v>
       </c>
       <c r="D15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;D4,月次固定費!$F$5:$F$17)</f>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;D4,月次固定費!$F$5:$F$19)</f>
         <v>106</v>
       </c>
       <c r="E15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;E4,月次固定費!$F$5:$F$17)</f>
-        <v>166</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;E4,月次固定費!$F$5:$F$19)</f>
+        <v>186</v>
       </c>
       <c r="F15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;F4,月次固定費!$F$5:$F$17)</f>
-        <v>166</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;F4,月次固定費!$F$5:$F$19)</f>
+        <v>186</v>
       </c>
       <c r="G15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;G4,月次固定費!$F$5:$F$17)</f>
-        <v>166</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;G4,月次固定費!$F$5:$F$19)</f>
+        <v>186</v>
       </c>
       <c r="H15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;H4,月次固定費!$F$5:$F$17)</f>
-        <v>226</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;H4,月次固定費!$F$5:$F$19)</f>
+        <v>271</v>
       </c>
       <c r="I15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;I4,月次固定費!$F$5:$F$17)</f>
-        <v>226</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;I4,月次固定費!$F$5:$F$19)</f>
+        <v>271</v>
       </c>
       <c r="J15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;J4,月次固定費!$F$5:$F$17)</f>
-        <v>226</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;J4,月次固定費!$F$5:$F$19)</f>
+        <v>271</v>
       </c>
       <c r="K15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;K4,月次固定費!$F$5:$F$17)</f>
-        <v>226</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;K4,月次固定費!$F$5:$F$19)</f>
+        <v>271</v>
       </c>
       <c r="L15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;L4,月次固定費!$F$5:$F$17)</f>
-        <v>226</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;L4,月次固定費!$F$5:$F$19)</f>
+        <v>271</v>
       </c>
       <c r="M15" s="22" t="n">
-        <f aca="false">SUMIF(月次固定費!$B$5:$B$17,"&lt;="&amp;M4,月次固定費!$F$5:$F$17)</f>
-        <v>226</v>
+        <f aca="false">SUMIF(月次固定費!$B$5:$B$19,"&lt;="&amp;M4,月次固定費!$F$5:$F$19)</f>
+        <v>271</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">B6*前提!$E$33</f>
@@ -6152,7 +6509,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">IF(B4&gt;=前提!$B$16,前提!$B$15*前提!$B$17/12,0)</f>
@@ -6205,7 +6562,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="20" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B18" s="23" t="n">
         <f aca="false">SUM(B14:B17)</f>
@@ -6221,44 +6578,44 @@
       </c>
       <c r="E18" s="23" t="n">
         <f aca="false">SUM(E14:E17)</f>
-        <v>193</v>
+        <v>213</v>
       </c>
       <c r="F18" s="23" t="n">
         <f aca="false">SUM(F14:F17)</f>
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="G18" s="23" t="n">
         <f aca="false">SUM(G14:G17)</f>
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="H18" s="23" t="n">
         <f aca="false">SUM(H14:H17)</f>
-        <v>297</v>
+        <v>342</v>
       </c>
       <c r="I18" s="23" t="n">
         <f aca="false">SUM(I14:I17)</f>
-        <v>297</v>
+        <v>342</v>
       </c>
       <c r="J18" s="23" t="n">
         <f aca="false">SUM(J14:J17)</f>
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="K18" s="23" t="n">
         <f aca="false">SUM(K14:K17)</f>
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="L18" s="23" t="n">
         <f aca="false">SUM(L14:L17)</f>
-        <v>341</v>
+        <v>386</v>
       </c>
       <c r="M18" s="23" t="n">
         <f aca="false">SUM(M14:M17)</f>
-        <v>341</v>
+        <v>386</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B20" s="23" t="n">
         <f aca="false">B12-B18</f>
@@ -6274,44 +6631,44 @@
       </c>
       <c r="E20" s="23" t="n">
         <f aca="false">E12-E18</f>
-        <v>-193</v>
+        <v>-213</v>
       </c>
       <c r="F20" s="23" t="n">
         <f aca="false">F12-F18</f>
-        <v>-167</v>
+        <v>-187</v>
       </c>
       <c r="G20" s="23" t="n">
         <f aca="false">G12-G18</f>
-        <v>-119</v>
+        <v>-139</v>
       </c>
       <c r="H20" s="23" t="n">
         <f aca="false">H12-H18</f>
-        <v>-201</v>
+        <v>-246</v>
       </c>
       <c r="I20" s="23" t="n">
         <f aca="false">I12-I18</f>
-        <v>-153</v>
+        <v>-198</v>
       </c>
       <c r="J20" s="23" t="n">
         <f aca="false">J12-J18</f>
-        <v>-175</v>
+        <v>-220</v>
       </c>
       <c r="K20" s="23" t="n">
         <f aca="false">K12-K18</f>
-        <v>-127</v>
+        <v>-172</v>
       </c>
       <c r="L20" s="23" t="n">
         <f aca="false">L12-L18</f>
-        <v>-149</v>
+        <v>-194</v>
       </c>
       <c r="M20" s="23" t="n">
         <f aca="false">M12-M18</f>
-        <v>-101</v>
+        <v>-146</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B21" s="30" t="n">
         <f aca="false">B20</f>
@@ -6327,53 +6684,53 @@
       </c>
       <c r="E21" s="30" t="n">
         <f aca="false">D21+E20</f>
-        <v>1492.35</v>
+        <v>1472.35</v>
       </c>
       <c r="F21" s="30" t="n">
         <f aca="false">E21+F20</f>
-        <v>1325.35</v>
+        <v>1285.35</v>
       </c>
       <c r="G21" s="30" t="n">
         <f aca="false">F21+G20</f>
-        <v>1206.35</v>
+        <v>1146.35</v>
       </c>
       <c r="H21" s="30" t="n">
         <f aca="false">G21+H20</f>
-        <v>1005.35</v>
+        <v>900.35</v>
       </c>
       <c r="I21" s="30" t="n">
         <f aca="false">H21+I20</f>
-        <v>852.35</v>
+        <v>702.35</v>
       </c>
       <c r="J21" s="30" t="n">
         <f aca="false">I21+J20</f>
-        <v>677.35</v>
+        <v>482.35</v>
       </c>
       <c r="K21" s="30" t="n">
         <f aca="false">J21+K20</f>
-        <v>550.35</v>
+        <v>310.35</v>
       </c>
       <c r="L21" s="30" t="n">
         <f aca="false">K21+L20</f>
-        <v>401.35</v>
+        <v>116.35</v>
       </c>
       <c r="M21" s="30" t="n">
         <f aca="false">L21+M20</f>
-        <v>300.35</v>
+        <v>-29.6500000000001</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B23" s="25" t="n">
         <f aca="false">MIN(B21:M21)</f>
-        <v>300.35</v>
+        <v>-29.6500000000001</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B24" s="20" t="str">
         <f aca="false">INDEX(B5:M5,MATCH(B23,B21:M21,0))</f>
@@ -6382,7 +6739,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B25" s="26" t="n">
         <f aca="false">SUM(B6:M6)</f>
@@ -6391,7 +6748,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B26" s="25" t="n">
         <f aca="false">SUM(B7:M7)</f>
@@ -6424,49 +6781,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B4" s="22" t="n">
         <f aca="false">初期費用!F17</f>
         <v>886.65</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B5" s="22" t="n">
-        <f aca="false">月次固定費!F18</f>
-        <v>226</v>
+        <f aca="false">月次固定費!F20</f>
+        <v>271</v>
       </c>
       <c r="C5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B6" s="31" t="n">
-        <f aca="false">月次固定費!F21</f>
-        <v>8.69230769230769</v>
+        <f aca="false">月次固定費!F23</f>
+        <v>10.4230769230769</v>
       </c>
       <c r="C6" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">前提!B14+前提!B15</f>
@@ -6476,19 +6833,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">資金繰り!B23</f>
-        <v>300.35</v>
+        <v>-29.6500000000001</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B10" s="6" t="str">
         <f aca="false">資金繰り!B24</f>
@@ -6498,73 +6855,73 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">資金繰り!M21</f>
-        <v>300.35</v>
+        <v>-29.6500000000001</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B13" s="22" t="n">
-        <f aca="false">月次固定費!F18*前提!B18</f>
-        <v>678</v>
+        <f aca="false">月次固定費!F20*前提!B18</f>
+        <v>813</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B14" s="25" t="n">
-        <f aca="false">MAX(0,月次固定費!F18*前提!B18-資金繰り!B23)</f>
-        <v>377.65</v>
+        <f aca="false">MAX(0,月次固定費!F20*前提!B18-資金繰り!B23)</f>
+        <v>842.65</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="B15" s="32" t="n">
         <f aca="false">B8+B14</f>
-        <v>3177.65</v>
+        <v>3642.65</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6572,12 +6929,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -6605,34 +6962,34 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="33" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>35</v>
@@ -6652,7 +7009,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>48</v>
@@ -6672,7 +7029,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>22</v>
@@ -6692,7 +7049,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>0</v>
@@ -6712,7 +7069,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>0.2</v>
@@ -6732,7 +7089,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="B10" s="15" t="n">
         <v>3</v>
@@ -6752,7 +7109,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B11" s="11" t="n">
         <v>720</v>
@@ -6772,7 +7129,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>0.6</v>
@@ -6792,7 +7149,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B13" s="11" t="n">
         <v>1100</v>
@@ -6812,7 +7169,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="B15" s="29" t="n">
         <f aca="false">B5*B6</f>
@@ -6837,7 +7194,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="B16" s="29" t="n">
         <f aca="false">B8</f>
@@ -6862,7 +7219,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="20" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B17" s="23" t="n">
         <f aca="false">B15+B16</f>
@@ -6887,7 +7244,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B18" s="29" t="n">
         <f aca="false">B5*B7+B8*B9</f>
@@ -6912,7 +7269,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="20" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="B19" s="23" t="n">
         <f aca="false">B17-B18</f>
@@ -6962,7 +7319,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="B21" s="29" t="n">
         <f aca="false">B10*B11*B12</f>
@@ -6987,7 +7344,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B22" s="29" t="n">
         <f aca="false">B13</f>
@@ -7012,7 +7369,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B23" s="23" t="n">
         <f aca="false">B21+B22</f>
@@ -7037,7 +7394,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="20" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B24" s="24" t="n">
         <f aca="false">B19-B23</f>
@@ -7062,7 +7419,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B25" s="34" t="n">
         <f aca="false">IF(B17=0,0,B24/B17)</f>
@@ -7087,7 +7444,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="B27" s="35" t="n">
         <f aca="false">IF(B17=0,0,B16/B17)</f>
@@ -7112,7 +7469,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B28" s="29" t="n">
         <f aca="false">IF(B10=0,0,B17/B10)</f>
@@ -7137,17 +7494,17 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>